<commit_message>
Atualização de ativos.xlsx e script
Adiciona universo dinâmico Bybit e configs de contexto
</commit_message>
<xml_diff>
--- a/ativos.xlsx
+++ b/ativos.xlsx
@@ -1,22 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\INVESTIMENTOS VARIAVEL\Bybit\bybit_setups\complementos\GitHub\bybit_setups\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E118378-A4CB-462D-8011-FFA246FEB3D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1B0280B-E961-443A-8119-28EC508648B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="PARES" sheetId="1" r:id="rId1"/>
+    <sheet name="CONFIG_UNIVERSO" sheetId="3" r:id="rId2"/>
+    <sheet name="CONFIG_REGIME" sheetId="4" r:id="rId3"/>
+    <sheet name="CONFIG_FORCA_RELATIVA" sheetId="5" r:id="rId4"/>
+    <sheet name="CONFIG_FUNDING_OI" sheetId="6" r:id="rId5"/>
+    <sheet name="CONFIG_GRID" sheetId="7" r:id="rId6"/>
+    <sheet name="EXCECOES_ATIVOS" sheetId="8" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$C$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PARES!$A$1:$C$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="819" uniqueCount="412">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="952" uniqueCount="516">
   <si>
     <t>Par</t>
   </si>
@@ -1272,13 +1278,325 @@
   </si>
   <si>
     <t>OPGUSDT</t>
+  </si>
+  <si>
+    <t>Parametro</t>
+  </si>
+  <si>
+    <t>Valor</t>
+  </si>
+  <si>
+    <t>Descricao</t>
+  </si>
+  <si>
+    <t>modo_universo</t>
+  </si>
+  <si>
+    <t>HIBRIDO</t>
+  </si>
+  <si>
+    <t>AUTO busca tudo na Bybit; MANUAL usa ativos.xlsx; HIBRIDO usa Bybit + exceções.</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>Categoria Bybit V5.</t>
+  </si>
+  <si>
+    <t>quote_coin</t>
+  </si>
+  <si>
+    <t>USDT</t>
+  </si>
+  <si>
+    <t>Moeda de cotação.</t>
+  </si>
+  <si>
+    <t>settle_coin</t>
+  </si>
+  <si>
+    <t>Moeda de liquidação.</t>
+  </si>
+  <si>
+    <t>contract_type</t>
+  </si>
+  <si>
+    <t>LinearPerpetual</t>
+  </si>
+  <si>
+    <t>Tipo de contrato.</t>
+  </si>
+  <si>
+    <t>min_age_days</t>
+  </si>
+  <si>
+    <t>Idade mínima desde listagem.</t>
+  </si>
+  <si>
+    <t>default_timeframes</t>
+  </si>
+  <si>
+    <t>240</t>
+  </si>
+  <si>
+    <t>Timeframes padrão para ativos automáticos. Ex.: 240 ou 120,240.</t>
+  </si>
+  <si>
+    <t>kline_limit</t>
+  </si>
+  <si>
+    <t>Quantidade de candles por par/timeframe.</t>
+  </si>
+  <si>
+    <t>min_turnover24h_usdt</t>
+  </si>
+  <si>
+    <t>Turnover financeiro mínimo em 24h.</t>
+  </si>
+  <si>
+    <t>max_spread_pct</t>
+  </si>
+  <si>
+    <t>Spread máximo bid/ask. 0,0005 = 0,05%.</t>
+  </si>
+  <si>
+    <t>min_open_interest_value</t>
+  </si>
+  <si>
+    <t>Open Interest Value mínimo.</t>
+  </si>
+  <si>
+    <t>orderbook_limit</t>
+  </si>
+  <si>
+    <t>Profundidade do book consultada.</t>
+  </si>
+  <si>
+    <t>min_depth_1pct_usdt</t>
+  </si>
+  <si>
+    <t>Profundidade mínima até 1% no lado mais fraco.</t>
+  </si>
+  <si>
+    <t>max_slippage_pct</t>
+  </si>
+  <si>
+    <t>Slippage estimado máximo. 0,003 = 0,30%.</t>
+  </si>
+  <si>
+    <t>capturar_orderbook</t>
+  </si>
+  <si>
+    <t>SIM</t>
+  </si>
+  <si>
+    <t>Capturar profundidade, imbalance e slippage estimado.</t>
+  </si>
+  <si>
+    <t>capturar_oi_historico</t>
+  </si>
+  <si>
+    <t>Capturar histórico de Open Interest.</t>
+  </si>
+  <si>
+    <t>capturar_funding_historico</t>
+  </si>
+  <si>
+    <t>Capturar histórico de funding para z-score.</t>
+  </si>
+  <si>
+    <t>capturar_long_short</t>
+  </si>
+  <si>
+    <t>Capturar long/short ratio.</t>
+  </si>
+  <si>
+    <t>adx_period</t>
+  </si>
+  <si>
+    <t>Período do ADX.</t>
+  </si>
+  <si>
+    <t>atr_period</t>
+  </si>
+  <si>
+    <t>Período do ATR para regime.</t>
+  </si>
+  <si>
+    <t>chop_period</t>
+  </si>
+  <si>
+    <t>Período do Choppiness Index.</t>
+  </si>
+  <si>
+    <t>er_period</t>
+  </si>
+  <si>
+    <t>Período do Efficiency Ratio.</t>
+  </si>
+  <si>
+    <t>bb_period</t>
+  </si>
+  <si>
+    <t>Período das Bandas de Bollinger.</t>
+  </si>
+  <si>
+    <t>bb_std</t>
+  </si>
+  <si>
+    <t>Desvio padrão das Bandas de Bollinger.</t>
+  </si>
+  <si>
+    <t>percentile_lookback</t>
+  </si>
+  <si>
+    <t>Janela para percentis de ATR/BB Width.</t>
+  </si>
+  <si>
+    <t>adx_min_trend</t>
+  </si>
+  <si>
+    <t>ADX mínimo para regime de tendência.</t>
+  </si>
+  <si>
+    <t>chop_max_trend</t>
+  </si>
+  <si>
+    <t>CHOP máximo para tendência.</t>
+  </si>
+  <si>
+    <t>er_min_trend</t>
+  </si>
+  <si>
+    <t>Efficiency Ratio mínimo.</t>
+  </si>
+  <si>
+    <t>atr_percentile_min</t>
+  </si>
+  <si>
+    <t>ATR percentil mínimo.</t>
+  </si>
+  <si>
+    <t>atr_percentile_max</t>
+  </si>
+  <si>
+    <t>ATR percentil máximo.</t>
+  </si>
+  <si>
+    <t>bb_width_percentile_compression</t>
+  </si>
+  <si>
+    <t>BB Width percentil abaixo disso indica compressão.</t>
+  </si>
+  <si>
+    <t>rs_short_window</t>
+  </si>
+  <si>
+    <t>Janela curta de retorno em candles.</t>
+  </si>
+  <si>
+    <t>rs_mid_window</t>
+  </si>
+  <si>
+    <t>Janela média de retorno em candles.</t>
+  </si>
+  <si>
+    <t>rs_long_window</t>
+  </si>
+  <si>
+    <t>Janela longa de retorno em candles.</t>
+  </si>
+  <si>
+    <t>rs_min_long</t>
+  </si>
+  <si>
+    <t>Rank mínimo para compra/long.</t>
+  </si>
+  <si>
+    <t>rs_max_short</t>
+  </si>
+  <si>
+    <t>Rank máximo para venda/short.</t>
+  </si>
+  <si>
+    <t>score_min_setup</t>
+  </si>
+  <si>
+    <t>Score mínimo para APROVADO_SCORE.</t>
+  </si>
+  <si>
+    <t>max_abs_funding_rate</t>
+  </si>
+  <si>
+    <t>Funding absoluto máximo. 0,003 = 0,30%.</t>
+  </si>
+  <si>
+    <t>max_funding_zscore</t>
+  </si>
+  <si>
+    <t>Z-score máximo de funding.</t>
+  </si>
+  <si>
+    <t>oi_interval</t>
+  </si>
+  <si>
+    <t>4h</t>
+  </si>
+  <si>
+    <t>Intervalo do Open Interest histórico.</t>
+  </si>
+  <si>
+    <t>account_ratio_period</t>
+  </si>
+  <si>
+    <t>Intervalo do long/short ratio.</t>
+  </si>
+  <si>
+    <t>api_sleep_s</t>
+  </si>
+  <si>
+    <t>Pausa entre chamadas REST públicas.</t>
+  </si>
+  <si>
+    <t>grid_spacing_pct</t>
+  </si>
+  <si>
+    <t>Espaçamento de referência para estimar número de grids. 0,005 = 0,50%.</t>
+  </si>
+  <si>
+    <t>Acao</t>
+  </si>
+  <si>
+    <t>Timeframes</t>
+  </si>
+  <si>
+    <t>Observacao</t>
+  </si>
+  <si>
+    <t>BTCUSDT</t>
+  </si>
+  <si>
+    <t>FORCAR_INCLUSAO</t>
+  </si>
+  <si>
+    <t>Exemplo: sempre analisar.</t>
+  </si>
+  <si>
+    <t>TOKENXYZUSDT</t>
+  </si>
+  <si>
+    <t>EXCLUIR</t>
+  </si>
+  <si>
+    <t>Exemplo: bloquear ativo manualmente.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1294,13 +1612,29 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0F766E"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -1327,17 +1661,23 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{3FE34418-C5A5-4AF1-A5F7-3EE7E148DFB4}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1640,12 +1980,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C409"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1656,7 +1996,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>385</v>
       </c>
@@ -1667,7 +2007,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>59</v>
       </c>
@@ -1678,7 +2018,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>372</v>
       </c>
@@ -1689,7 +2029,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1700,7 +2040,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1711,7 +2051,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>60</v>
       </c>
@@ -1722,7 +2062,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>373</v>
       </c>
@@ -1733,7 +2073,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>61</v>
       </c>
@@ -1744,7 +2084,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -1755,7 +2095,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>386</v>
       </c>
@@ -1766,7 +2106,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>63</v>
       </c>
@@ -1777,7 +2117,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>64</v>
       </c>
@@ -1788,7 +2128,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>65</v>
       </c>
@@ -1799,7 +2139,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>66</v>
       </c>
@@ -1810,7 +2150,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>67</v>
       </c>
@@ -1821,7 +2161,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>6</v>
       </c>
@@ -1832,7 +2172,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>68</v>
       </c>
@@ -1843,7 +2183,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>69</v>
       </c>
@@ -1854,7 +2194,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>70</v>
       </c>
@@ -1865,7 +2205,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>71</v>
       </c>
@@ -1876,7 +2216,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>72</v>
       </c>
@@ -1887,7 +2227,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>387</v>
       </c>
@@ -1898,7 +2238,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>73</v>
       </c>
@@ -1909,7 +2249,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>400</v>
       </c>
@@ -1920,7 +2260,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>74</v>
       </c>
@@ -1931,7 +2271,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>75</v>
       </c>
@@ -1942,7 +2282,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>7</v>
       </c>
@@ -1953,7 +2293,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>76</v>
       </c>
@@ -1964,7 +2304,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>388</v>
       </c>
@@ -1975,7 +2315,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>77</v>
       </c>
@@ -1986,7 +2326,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>78</v>
       </c>
@@ -1997,7 +2337,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>79</v>
       </c>
@@ -2008,7 +2348,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>8</v>
       </c>
@@ -2019,7 +2359,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>9</v>
       </c>
@@ -2030,7 +2370,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>389</v>
       </c>
@@ -2041,7 +2381,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>80</v>
       </c>
@@ -2052,7 +2392,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>81</v>
       </c>
@@ -2063,7 +2403,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>10</v>
       </c>
@@ -2074,7 +2414,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>390</v>
       </c>
@@ -2085,7 +2425,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>83</v>
       </c>
@@ -2096,7 +2436,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>82</v>
       </c>
@@ -2107,7 +2447,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>84</v>
       </c>
@@ -2118,7 +2458,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>374</v>
       </c>
@@ -2129,7 +2469,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>391</v>
       </c>
@@ -2140,7 +2480,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>392</v>
       </c>
@@ -2151,7 +2491,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>85</v>
       </c>
@@ -2162,7 +2502,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>86</v>
       </c>
@@ -2173,7 +2513,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>87</v>
       </c>
@@ -2184,7 +2524,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>393</v>
       </c>
@@ -2195,7 +2535,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>88</v>
       </c>
@@ -2206,7 +2546,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>62</v>
       </c>
@@ -2217,7 +2557,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>89</v>
       </c>
@@ -2228,7 +2568,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>11</v>
       </c>
@@ -2239,7 +2579,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>394</v>
       </c>
@@ -2250,7 +2590,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>90</v>
       </c>
@@ -2261,7 +2601,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>91</v>
       </c>
@@ -2272,7 +2612,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>92</v>
       </c>
@@ -2283,7 +2623,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>93</v>
       </c>
@@ -2294,7 +2634,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>94</v>
       </c>
@@ -2305,7 +2645,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>95</v>
       </c>
@@ -2316,7 +2656,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>97</v>
       </c>
@@ -2327,7 +2667,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>98</v>
       </c>
@@ -2338,7 +2678,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>99</v>
       </c>
@@ -2349,7 +2689,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>96</v>
       </c>
@@ -2360,7 +2700,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>100</v>
       </c>
@@ -2371,7 +2711,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>101</v>
       </c>
@@ -2382,7 +2722,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>102</v>
       </c>
@@ -2393,7 +2733,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>103</v>
       </c>
@@ -2404,7 +2744,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>397</v>
       </c>
@@ -2415,7 +2755,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>104</v>
       </c>
@@ -2426,7 +2766,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>105</v>
       </c>
@@ -2437,7 +2777,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>106</v>
       </c>
@@ -2448,7 +2788,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>12</v>
       </c>
@@ -2459,7 +2799,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>107</v>
       </c>
@@ -2470,7 +2810,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>375</v>
       </c>
@@ -2481,7 +2821,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>402</v>
       </c>
@@ -2492,7 +2832,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>108</v>
       </c>
@@ -2503,7 +2843,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>109</v>
       </c>
@@ -2514,7 +2854,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>13</v>
       </c>
@@ -2525,7 +2865,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>110</v>
       </c>
@@ -2536,7 +2876,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>111</v>
       </c>
@@ -2547,7 +2887,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>112</v>
       </c>
@@ -2558,7 +2898,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>14</v>
       </c>
@@ -2569,7 +2909,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>113</v>
       </c>
@@ -2580,7 +2920,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>15</v>
       </c>
@@ -2591,7 +2931,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>114</v>
       </c>
@@ -2602,7 +2942,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>396</v>
       </c>
@@ -2613,7 +2953,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>409</v>
       </c>
@@ -2624,7 +2964,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>116</v>
       </c>
@@ -2635,7 +2975,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>117</v>
       </c>
@@ -2646,7 +2986,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>118</v>
       </c>
@@ -2657,7 +2997,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>119</v>
       </c>
@@ -2668,7 +3008,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>120</v>
       </c>
@@ -2679,7 +3019,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>121</v>
       </c>
@@ -2690,7 +3030,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>122</v>
       </c>
@@ -2701,7 +3041,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>123</v>
       </c>
@@ -2712,7 +3052,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>124</v>
       </c>
@@ -2723,7 +3063,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>125</v>
       </c>
@@ -2734,7 +3074,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>126</v>
       </c>
@@ -2745,7 +3085,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>376</v>
       </c>
@@ -2756,7 +3096,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>127</v>
       </c>
@@ -2767,7 +3107,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>408</v>
       </c>
@@ -2778,7 +3118,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>16</v>
       </c>
@@ -2789,7 +3129,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>128</v>
       </c>
@@ -2800,7 +3140,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>17</v>
       </c>
@@ -2811,7 +3151,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>18</v>
       </c>
@@ -2822,7 +3162,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>129</v>
       </c>
@@ -2833,7 +3173,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>131</v>
       </c>
@@ -2844,7 +3184,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>130</v>
       </c>
@@ -2855,7 +3195,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>132</v>
       </c>
@@ -2866,7 +3206,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>133</v>
       </c>
@@ -2877,7 +3217,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>115</v>
       </c>
@@ -2888,7 +3228,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>134</v>
       </c>
@@ -2899,7 +3239,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>135</v>
       </c>
@@ -2910,7 +3250,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>136</v>
       </c>
@@ -2921,7 +3261,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>137</v>
       </c>
@@ -2932,7 +3272,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>138</v>
       </c>
@@ -2943,7 +3283,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>139</v>
       </c>
@@ -2954,7 +3294,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>140</v>
       </c>
@@ -2965,7 +3305,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>141</v>
       </c>
@@ -2976,7 +3316,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>19</v>
       </c>
@@ -2987,7 +3327,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>142</v>
       </c>
@@ -2998,7 +3338,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>143</v>
       </c>
@@ -3009,7 +3349,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>144</v>
       </c>
@@ -3020,7 +3360,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>145</v>
       </c>
@@ -3031,7 +3371,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>146</v>
       </c>
@@ -3042,7 +3382,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>147</v>
       </c>
@@ -3053,7 +3393,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>403</v>
       </c>
@@ -3064,7 +3404,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>148</v>
       </c>
@@ -3075,7 +3415,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>149</v>
       </c>
@@ -3086,7 +3426,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>150</v>
       </c>
@@ -3097,7 +3437,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>20</v>
       </c>
@@ -3108,7 +3448,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>151</v>
       </c>
@@ -3119,7 +3459,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>152</v>
       </c>
@@ -3130,7 +3470,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>153</v>
       </c>
@@ -3141,7 +3481,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>154</v>
       </c>
@@ -3152,7 +3492,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>155</v>
       </c>
@@ -3163,7 +3503,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>156</v>
       </c>
@@ -3174,7 +3514,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>157</v>
       </c>
@@ -3185,7 +3525,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>158</v>
       </c>
@@ -3196,7 +3536,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>21</v>
       </c>
@@ -3207,7 +3547,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>410</v>
       </c>
@@ -3218,7 +3558,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>22</v>
       </c>
@@ -3229,7 +3569,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>399</v>
       </c>
@@ -3240,7 +3580,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>159</v>
       </c>
@@ -3251,7 +3591,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>160</v>
       </c>
@@ -3262,7 +3602,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>161</v>
       </c>
@@ -3273,7 +3613,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>162</v>
       </c>
@@ -3284,7 +3624,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>163</v>
       </c>
@@ -3295,7 +3635,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>164</v>
       </c>
@@ -3306,7 +3646,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>405</v>
       </c>
@@ -3317,7 +3657,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>165</v>
       </c>
@@ -3328,7 +3668,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>23</v>
       </c>
@@ -3339,7 +3679,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>24</v>
       </c>
@@ -3350,7 +3690,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>166</v>
       </c>
@@ -3361,7 +3701,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>395</v>
       </c>
@@ -3372,7 +3712,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>167</v>
       </c>
@@ -3383,7 +3723,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>168</v>
       </c>
@@ -3394,7 +3734,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>25</v>
       </c>
@@ -3405,7 +3745,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>169</v>
       </c>
@@ -3416,7 +3756,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>170</v>
       </c>
@@ -3427,7 +3767,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>171</v>
       </c>
@@ -3438,7 +3778,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>172</v>
       </c>
@@ -3449,7 +3789,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>173</v>
       </c>
@@ -3460,7 +3800,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>174</v>
       </c>
@@ -3471,7 +3811,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>175</v>
       </c>
@@ -3482,7 +3822,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>176</v>
       </c>
@@ -3493,7 +3833,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>177</v>
       </c>
@@ -3504,7 +3844,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>179</v>
       </c>
@@ -3515,7 +3855,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>180</v>
       </c>
@@ -3526,7 +3866,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>181</v>
       </c>
@@ -3537,7 +3877,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>182</v>
       </c>
@@ -3548,7 +3888,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>183</v>
       </c>
@@ -3559,7 +3899,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>184</v>
       </c>
@@ -3570,7 +3910,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>185</v>
       </c>
@@ -3581,7 +3921,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>186</v>
       </c>
@@ -3592,7 +3932,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>187</v>
       </c>
@@ -3603,7 +3943,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>188</v>
       </c>
@@ -3614,7 +3954,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>178</v>
       </c>
@@ -3625,7 +3965,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>190</v>
       </c>
@@ -3636,7 +3976,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>189</v>
       </c>
@@ -3647,7 +3987,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>191</v>
       </c>
@@ -3658,7 +3998,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>377</v>
       </c>
@@ -3669,7 +4009,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>192</v>
       </c>
@@ -3680,7 +4020,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>193</v>
       </c>
@@ -3691,7 +4031,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>194</v>
       </c>
@@ -3702,7 +4042,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>195</v>
       </c>
@@ -3713,7 +4053,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>196</v>
       </c>
@@ -3724,7 +4064,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>197</v>
       </c>
@@ -3735,7 +4075,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>199</v>
       </c>
@@ -3746,7 +4086,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>200</v>
       </c>
@@ -3757,7 +4097,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>201</v>
       </c>
@@ -3768,7 +4108,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>198</v>
       </c>
@@ -3779,7 +4119,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>202</v>
       </c>
@@ -3790,7 +4130,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>26</v>
       </c>
@@ -3801,7 +4141,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>203</v>
       </c>
@@ -3812,7 +4152,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>204</v>
       </c>
@@ -3823,7 +4163,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>27</v>
       </c>
@@ -3834,7 +4174,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>28</v>
       </c>
@@ -3845,7 +4185,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>205</v>
       </c>
@@ -3856,7 +4196,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="202" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>206</v>
       </c>
@@ -3867,7 +4207,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="203" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>29</v>
       </c>
@@ -3878,7 +4218,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="204" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>207</v>
       </c>
@@ -3889,7 +4229,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="205" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>378</v>
       </c>
@@ -3900,7 +4240,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="206" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>30</v>
       </c>
@@ -3911,7 +4251,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="207" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>208</v>
       </c>
@@ -3922,7 +4262,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="208" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>209</v>
       </c>
@@ -3933,7 +4273,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="209" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>210</v>
       </c>
@@ -3944,7 +4284,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="210" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>211</v>
       </c>
@@ -3955,7 +4295,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="211" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>398</v>
       </c>
@@ -3966,7 +4306,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="212" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>31</v>
       </c>
@@ -3977,7 +4317,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="213" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>212</v>
       </c>
@@ -3988,7 +4328,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="214" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>213</v>
       </c>
@@ -3999,7 +4339,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="215" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>214</v>
       </c>
@@ -4010,7 +4350,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="216" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>215</v>
       </c>
@@ -4021,7 +4361,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>216</v>
       </c>
@@ -4032,7 +4372,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="218" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>217</v>
       </c>
@@ -4043,7 +4383,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="219" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>218</v>
       </c>
@@ -4054,7 +4394,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="220" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>220</v>
       </c>
@@ -4065,7 +4405,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="221" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>404</v>
       </c>
@@ -4076,7 +4416,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="222" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>32</v>
       </c>
@@ -4087,7 +4427,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>221</v>
       </c>
@@ -4098,7 +4438,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="224" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>222</v>
       </c>
@@ -4109,7 +4449,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="225" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>224</v>
       </c>
@@ -4120,7 +4460,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="226" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>223</v>
       </c>
@@ -4131,7 +4471,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="227" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>225</v>
       </c>
@@ -4142,7 +4482,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="228" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>227</v>
       </c>
@@ -4153,7 +4493,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="229" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>228</v>
       </c>
@@ -4164,7 +4504,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="230" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>229</v>
       </c>
@@ -4175,7 +4515,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="231" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>230</v>
       </c>
@@ -4186,7 +4526,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="232" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>226</v>
       </c>
@@ -4197,7 +4537,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="233" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>33</v>
       </c>
@@ -4208,7 +4548,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="234" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>231</v>
       </c>
@@ -4219,7 +4559,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="235" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>232</v>
       </c>
@@ -4230,7 +4570,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="236" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>34</v>
       </c>
@@ -4241,7 +4581,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="237" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>233</v>
       </c>
@@ -4252,7 +4592,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="238" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>35</v>
       </c>
@@ -4263,7 +4603,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="239" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>36</v>
       </c>
@@ -4274,7 +4614,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="240" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>234</v>
       </c>
@@ -4285,7 +4625,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="241" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>235</v>
       </c>
@@ -4296,7 +4636,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="242" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>236</v>
       </c>
@@ -4307,7 +4647,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="243" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>237</v>
       </c>
@@ -4318,7 +4658,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="244" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>219</v>
       </c>
@@ -4329,7 +4669,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="245" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>384</v>
       </c>
@@ -4340,7 +4680,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="246" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>37</v>
       </c>
@@ -4351,7 +4691,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="247" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>238</v>
       </c>
@@ -4362,7 +4702,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="248" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>239</v>
       </c>
@@ -4373,7 +4713,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="249" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>240</v>
       </c>
@@ -4384,7 +4724,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="250" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>241</v>
       </c>
@@ -4395,7 +4735,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="251" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>401</v>
       </c>
@@ -4406,7 +4746,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="252" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>38</v>
       </c>
@@ -4417,7 +4757,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="253" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
         <v>242</v>
       </c>
@@ -4428,7 +4768,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="254" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>244</v>
       </c>
@@ -4439,7 +4779,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="255" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>243</v>
       </c>
@@ -4450,7 +4790,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="256" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>39</v>
       </c>
@@ -4461,7 +4801,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="257" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>245</v>
       </c>
@@ -4472,7 +4812,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="258" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
         <v>246</v>
       </c>
@@ -4483,7 +4823,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="259" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
         <v>411</v>
       </c>
@@ -4494,7 +4834,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="260" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>40</v>
       </c>
@@ -4505,7 +4845,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="261" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>247</v>
       </c>
@@ -4516,7 +4856,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="262" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>41</v>
       </c>
@@ -4527,7 +4867,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="263" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
         <v>248</v>
       </c>
@@ -4538,7 +4878,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="264" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>249</v>
       </c>
@@ -4549,7 +4889,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="265" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>250</v>
       </c>
@@ -4560,7 +4900,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="266" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
         <v>251</v>
       </c>
@@ -4571,7 +4911,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="267" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
         <v>252</v>
       </c>
@@ -4582,7 +4922,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="268" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
         <v>42</v>
       </c>
@@ -4593,7 +4933,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="269" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
         <v>253</v>
       </c>
@@ -4604,7 +4944,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="270" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A270" t="s">
         <v>254</v>
       </c>
@@ -4615,7 +4955,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="271" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
         <v>406</v>
       </c>
@@ -4626,7 +4966,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="272" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A272" t="s">
         <v>255</v>
       </c>
@@ -4637,7 +4977,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="273" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
         <v>256</v>
       </c>
@@ -4648,7 +4988,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="274" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
         <v>257</v>
       </c>
@@ -4659,7 +4999,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="275" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
         <v>258</v>
       </c>
@@ -4670,7 +5010,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="276" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A276" t="s">
         <v>259</v>
       </c>
@@ -4681,7 +5021,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="277" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A277" t="s">
         <v>260</v>
       </c>
@@ -4692,7 +5032,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="278" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
         <v>261</v>
       </c>
@@ -4703,7 +5043,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="279" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
         <v>43</v>
       </c>
@@ -4714,7 +5054,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="280" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
         <v>262</v>
       </c>
@@ -4725,7 +5065,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="281" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
         <v>263</v>
       </c>
@@ -4736,7 +5076,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="282" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
         <v>264</v>
       </c>
@@ -4747,7 +5087,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="283" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
         <v>265</v>
       </c>
@@ -4758,7 +5098,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="284" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
         <v>266</v>
       </c>
@@ -4769,7 +5109,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="285" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
         <v>267</v>
       </c>
@@ -4780,7 +5120,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="286" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
         <v>379</v>
       </c>
@@ -4791,7 +5131,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="287" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
         <v>268</v>
       </c>
@@ -4802,7 +5142,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="288" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A288" t="s">
         <v>44</v>
       </c>
@@ -4813,7 +5153,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="289" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A289" t="s">
         <v>269</v>
       </c>
@@ -4824,7 +5164,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="290" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A290" t="s">
         <v>270</v>
       </c>
@@ -4835,7 +5175,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="291" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A291" t="s">
         <v>271</v>
       </c>
@@ -4846,7 +5186,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="292" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A292" t="s">
         <v>272</v>
       </c>
@@ -4857,7 +5197,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="293" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A293" t="s">
         <v>273</v>
       </c>
@@ -4868,7 +5208,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="294" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A294" t="s">
         <v>274</v>
       </c>
@@ -4879,7 +5219,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="295" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A295" t="s">
         <v>275</v>
       </c>
@@ -4890,7 +5230,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="296" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A296" t="s">
         <v>276</v>
       </c>
@@ -4901,7 +5241,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="297" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A297" t="s">
         <v>277</v>
       </c>
@@ -4912,7 +5252,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="298" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A298" t="s">
         <v>278</v>
       </c>
@@ -4923,7 +5263,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="299" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
         <v>380</v>
       </c>
@@ -4934,7 +5274,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="300" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A300" t="s">
         <v>279</v>
       </c>
@@ -4945,7 +5285,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="301" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
         <v>280</v>
       </c>
@@ -4956,7 +5296,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="302" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
         <v>281</v>
       </c>
@@ -4967,7 +5307,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="303" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
         <v>45</v>
       </c>
@@ -4978,7 +5318,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="304" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
         <v>282</v>
       </c>
@@ -4989,7 +5329,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="305" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
         <v>284</v>
       </c>
@@ -5000,7 +5340,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="306" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
         <v>285</v>
       </c>
@@ -5011,7 +5351,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="307" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>286</v>
       </c>
@@ -5022,7 +5362,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="308" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
         <v>287</v>
       </c>
@@ -5033,7 +5373,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="309" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A309" t="s">
         <v>290</v>
       </c>
@@ -5044,7 +5384,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="310" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A310" t="s">
         <v>289</v>
       </c>
@@ -5055,7 +5395,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="311" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A311" t="s">
         <v>288</v>
       </c>
@@ -5066,7 +5406,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="312" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A312" t="s">
         <v>291</v>
       </c>
@@ -5077,7 +5417,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="313" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A313" t="s">
         <v>292</v>
       </c>
@@ -5088,7 +5428,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="314" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A314" t="s">
         <v>46</v>
       </c>
@@ -5099,7 +5439,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="315" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A315" t="s">
         <v>293</v>
       </c>
@@ -5110,7 +5450,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="316" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A316" t="s">
         <v>294</v>
       </c>
@@ -5121,7 +5461,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="317" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A317" t="s">
         <v>295</v>
       </c>
@@ -5132,7 +5472,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="318" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A318" t="s">
         <v>296</v>
       </c>
@@ -5143,7 +5483,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="319" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A319" t="s">
         <v>47</v>
       </c>
@@ -5154,7 +5494,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="320" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A320" t="s">
         <v>297</v>
       </c>
@@ -5165,7 +5505,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="321" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A321" t="s">
         <v>48</v>
       </c>
@@ -5176,7 +5516,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="322" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A322" t="s">
         <v>298</v>
       </c>
@@ -5187,7 +5527,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="323" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A323" t="s">
         <v>299</v>
       </c>
@@ -5198,7 +5538,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="324" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A324" t="s">
         <v>300</v>
       </c>
@@ -5209,7 +5549,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="325" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A325" t="s">
         <v>301</v>
       </c>
@@ -5220,7 +5560,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="326" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A326" t="s">
         <v>302</v>
       </c>
@@ -5231,7 +5571,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="327" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A327" t="s">
         <v>303</v>
       </c>
@@ -5242,7 +5582,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="328" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A328" t="s">
         <v>49</v>
       </c>
@@ -5253,7 +5593,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="329" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A329" t="s">
         <v>304</v>
       </c>
@@ -5264,7 +5604,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="330" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A330" t="s">
         <v>305</v>
       </c>
@@ -5275,7 +5615,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="331" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A331" t="s">
         <v>306</v>
       </c>
@@ -5286,7 +5626,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="332" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A332" t="s">
         <v>307</v>
       </c>
@@ -5297,7 +5637,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="333" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A333" t="s">
         <v>309</v>
       </c>
@@ -5308,7 +5648,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="334" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A334" t="s">
         <v>308</v>
       </c>
@@ -5319,7 +5659,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="335" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A335" t="s">
         <v>310</v>
       </c>
@@ -5330,7 +5670,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="336" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A336" t="s">
         <v>311</v>
       </c>
@@ -5341,7 +5681,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="337" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A337" t="s">
         <v>312</v>
       </c>
@@ -5352,7 +5692,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="338" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A338" t="s">
         <v>313</v>
       </c>
@@ -5363,7 +5703,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="339" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A339" t="s">
         <v>314</v>
       </c>
@@ -5374,7 +5714,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="340" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A340" t="s">
         <v>283</v>
       </c>
@@ -5385,7 +5725,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="341" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A341" t="s">
         <v>315</v>
       </c>
@@ -5396,7 +5736,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="342" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A342" t="s">
         <v>316</v>
       </c>
@@ -5407,7 +5747,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="343" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A343" t="s">
         <v>317</v>
       </c>
@@ -5418,7 +5758,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="344" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A344" t="s">
         <v>320</v>
       </c>
@@ -5429,7 +5769,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="345" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A345" t="s">
         <v>381</v>
       </c>
@@ -5440,7 +5780,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="346" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A346" t="s">
         <v>321</v>
       </c>
@@ -5451,7 +5791,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="347" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A347" t="s">
         <v>319</v>
       </c>
@@ -5462,7 +5802,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="348" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A348" t="s">
         <v>323</v>
       </c>
@@ -5473,7 +5813,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="349" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A349" t="s">
         <v>322</v>
       </c>
@@ -5484,7 +5824,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="350" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A350" t="s">
         <v>324</v>
       </c>
@@ -5495,7 +5835,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="351" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A351" t="s">
         <v>325</v>
       </c>
@@ -5506,7 +5846,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="352" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A352" t="s">
         <v>326</v>
       </c>
@@ -5517,7 +5857,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="353" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A353" t="s">
         <v>50</v>
       </c>
@@ -5528,7 +5868,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="354" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A354" t="s">
         <v>51</v>
       </c>
@@ -5539,7 +5879,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="355" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A355" t="s">
         <v>327</v>
       </c>
@@ -5550,7 +5890,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="356" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A356" t="s">
         <v>328</v>
       </c>
@@ -5561,7 +5901,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="357" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A357" t="s">
         <v>329</v>
       </c>
@@ -5572,7 +5912,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="358" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A358" t="s">
         <v>318</v>
       </c>
@@ -5583,7 +5923,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="359" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A359" t="s">
         <v>330</v>
       </c>
@@ -5594,7 +5934,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="360" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A360" t="s">
         <v>331</v>
       </c>
@@ -5605,7 +5945,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="361" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A361" t="s">
         <v>332</v>
       </c>
@@ -5616,7 +5956,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="362" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A362" t="s">
         <v>333</v>
       </c>
@@ -5627,7 +5967,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="363" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A363" t="s">
         <v>334</v>
       </c>
@@ -5638,7 +5978,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="364" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A364" t="s">
         <v>335</v>
       </c>
@@ -5649,7 +5989,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="365" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A365" t="s">
         <v>336</v>
       </c>
@@ -5660,7 +6000,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="366" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A366" t="s">
         <v>337</v>
       </c>
@@ -5671,7 +6011,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="367" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A367" t="s">
         <v>338</v>
       </c>
@@ -5682,7 +6022,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="368" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A368" t="s">
         <v>339</v>
       </c>
@@ -5693,7 +6033,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="369" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A369" t="s">
         <v>340</v>
       </c>
@@ -5704,7 +6044,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="370" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A370" t="s">
         <v>341</v>
       </c>
@@ -5715,7 +6055,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="371" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A371" t="s">
         <v>343</v>
       </c>
@@ -5726,7 +6066,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="372" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A372" t="s">
         <v>342</v>
       </c>
@@ -5737,7 +6077,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="373" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A373" t="s">
         <v>344</v>
       </c>
@@ -5748,7 +6088,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="374" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A374" t="s">
         <v>345</v>
       </c>
@@ -5759,7 +6099,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="375" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A375" t="s">
         <v>346</v>
       </c>
@@ -5770,7 +6110,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="376" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A376" t="s">
         <v>347</v>
       </c>
@@ -5781,7 +6121,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="377" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A377" t="s">
         <v>348</v>
       </c>
@@ -5792,7 +6132,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="378" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A378" t="s">
         <v>350</v>
       </c>
@@ -5803,7 +6143,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="379" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A379" t="s">
         <v>383</v>
       </c>
@@ -5814,7 +6154,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="380" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A380" t="s">
         <v>382</v>
       </c>
@@ -5825,7 +6165,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="381" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A381" t="s">
         <v>351</v>
       </c>
@@ -5836,7 +6176,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="382" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A382" t="s">
         <v>52</v>
       </c>
@@ -5847,7 +6187,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="383" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A383" t="s">
         <v>352</v>
       </c>
@@ -5858,7 +6198,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="384" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A384" t="s">
         <v>353</v>
       </c>
@@ -5869,7 +6209,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="385" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A385" t="s">
         <v>349</v>
       </c>
@@ -5880,7 +6220,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="386" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A386" t="s">
         <v>354</v>
       </c>
@@ -5891,7 +6231,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="387" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A387" t="s">
         <v>355</v>
       </c>
@@ -5902,7 +6242,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="388" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A388" t="s">
         <v>53</v>
       </c>
@@ -5913,7 +6253,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="389" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A389" t="s">
         <v>356</v>
       </c>
@@ -5924,7 +6264,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="390" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A390" t="s">
         <v>357</v>
       </c>
@@ -5935,7 +6275,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="391" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A391" t="s">
         <v>54</v>
       </c>
@@ -5946,7 +6286,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="392" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A392" t="s">
         <v>358</v>
       </c>
@@ -5957,7 +6297,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="393" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A393" t="s">
         <v>55</v>
       </c>
@@ -5968,7 +6308,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="394" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A394" t="s">
         <v>359</v>
       </c>
@@ -5979,7 +6319,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="395" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A395" t="s">
         <v>360</v>
       </c>
@@ -5990,7 +6330,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="396" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A396" t="s">
         <v>361</v>
       </c>
@@ -6001,7 +6341,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="397" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A397" t="s">
         <v>362</v>
       </c>
@@ -6012,7 +6352,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="398" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A398" t="s">
         <v>363</v>
       </c>
@@ -6023,7 +6363,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="399" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A399" t="s">
         <v>364</v>
       </c>
@@ -6034,7 +6374,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="400" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A400" t="s">
         <v>365</v>
       </c>
@@ -6045,7 +6385,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="401" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A401" t="s">
         <v>56</v>
       </c>
@@ -6056,7 +6396,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="402" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A402" t="s">
         <v>366</v>
       </c>
@@ -6067,7 +6407,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="403" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="403" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A403" t="s">
         <v>367</v>
       </c>
@@ -6078,7 +6418,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="404" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A404" t="s">
         <v>368</v>
       </c>
@@ -6089,7 +6429,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="405" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="405" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A405" t="s">
         <v>407</v>
       </c>
@@ -6100,7 +6440,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="406" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="406" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A406" t="s">
         <v>369</v>
       </c>
@@ -6111,7 +6451,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="407" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="407" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A407" t="s">
         <v>370</v>
       </c>
@@ -6122,7 +6462,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="408" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="408" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A408" t="s">
         <v>371</v>
       </c>
@@ -6133,7 +6473,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="409" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="409" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A409" t="s">
         <v>57</v>
       </c>
@@ -6155,4 +6495,703 @@
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93F0B986-6F00-4898-AAF8-4225C5C7F5F4}">
+  <dimension ref="A1:C19"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="28" style="3" customWidth="1"/>
+    <col min="2" max="2" width="20" style="3" customWidth="1"/>
+    <col min="3" max="3" width="70" style="3" customWidth="1"/>
+    <col min="4" max="16384" width="8.88671875" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>418</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>425</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>426</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="B7" s="3">
+        <v>90</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="B9" s="3">
+        <v>200</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="B10" s="3">
+        <v>10000000</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>437</v>
+      </c>
+      <c r="B11" s="3">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>439</v>
+      </c>
+      <c r="B12" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="B13" s="3">
+        <v>200</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="B14" s="3">
+        <v>250000</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="B15" s="3">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>455</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AD8DA9F-2545-4FA1-99BD-09F9BD908DA4}">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="28" style="3" customWidth="1"/>
+    <col min="2" max="2" width="20" style="3" customWidth="1"/>
+    <col min="3" max="3" width="70" style="3" customWidth="1"/>
+    <col min="4" max="16384" width="8.88671875" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>456</v>
+      </c>
+      <c r="B2" s="3">
+        <v>14</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="B3" s="3">
+        <v>14</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="B4" s="3">
+        <v>14</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>462</v>
+      </c>
+      <c r="B5" s="3">
+        <v>10</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>464</v>
+      </c>
+      <c r="B6" s="3">
+        <v>20</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>466</v>
+      </c>
+      <c r="B7" s="3">
+        <v>2</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>468</v>
+      </c>
+      <c r="B8" s="3">
+        <v>90</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>470</v>
+      </c>
+      <c r="B9" s="3">
+        <v>18</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="B10" s="3">
+        <v>55</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>474</v>
+      </c>
+      <c r="B11" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>476</v>
+      </c>
+      <c r="B12" s="3">
+        <v>25</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="B13" s="3">
+        <v>85</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="B14" s="3">
+        <v>20</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>481</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2959A29D-B2C8-4AE1-B616-61180D6215F2}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="28" style="3" customWidth="1"/>
+    <col min="2" max="2" width="20" style="3" customWidth="1"/>
+    <col min="3" max="3" width="70" style="3" customWidth="1"/>
+    <col min="4" max="16384" width="8.88671875" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="B2" s="3">
+        <v>3</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="B3" s="3">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="B4" s="3">
+        <v>12</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>488</v>
+      </c>
+      <c r="B5" s="3">
+        <v>65</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="B6" s="3">
+        <v>35</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="B7" s="3">
+        <v>70</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>493</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BB6560A-5865-43EC-BBFA-28BB0B0E8C87}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="28" style="3" customWidth="1"/>
+    <col min="2" max="2" width="20" style="3" customWidth="1"/>
+    <col min="3" max="3" width="70" style="3" customWidth="1"/>
+    <col min="4" max="16384" width="8.88671875" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="B2" s="3">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="B3" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>498</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>501</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="B6" s="3">
+        <v>0.08</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>504</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A338FB6F-4D01-4F24-AC37-909EB973780A}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="28" style="3" customWidth="1"/>
+    <col min="2" max="2" width="20" style="3" customWidth="1"/>
+    <col min="3" max="3" width="70" style="3" customWidth="1"/>
+    <col min="4" max="16384" width="8.88671875" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="B2" s="3">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>506</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EDA6476-619C-437C-94BC-2AF48BA6BE85}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18" style="3" customWidth="1"/>
+    <col min="2" max="2" width="20" style="3" customWidth="1"/>
+    <col min="3" max="3" width="18" style="3" customWidth="1"/>
+    <col min="4" max="4" width="12" style="3" customWidth="1"/>
+    <col min="5" max="5" width="60" style="3" customWidth="1"/>
+    <col min="6" max="16384" width="8.88671875" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>507</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>508</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>513</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>514</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>515</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" sqref="B2:B500" xr:uid="{89E22ECE-CA94-4B55-B0BE-434F5CBBD119}">
+      <formula1>"AUTO,FORCAR_INCLUSAO,EXCLUIR"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>